<commit_message>
29.09. Sve komitovano jer sam ostao sam
</commit_message>
<xml_diff>
--- a/testdata/configurationTST/execute.xlsx
+++ b/testdata/configurationTST/execute.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21216" windowHeight="8964"/>
+    <workbookView windowWidth="28800" windowHeight="12240"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$186</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1366" uniqueCount="380">
   <si>
     <t>App</t>
   </si>
@@ -81,21 +81,21 @@
     <t>C70780</t>
   </si>
   <si>
+    <t>Product_Summary_Sorting_on_the_Product_Summary_[ANDROID]</t>
+  </si>
+  <si>
+    <t>C70781</t>
+  </si>
+  <si>
+    <t>Product_Summary-Edit_Product_view-edit_name_of_account-invalid_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70782</t>
+  </si>
+  <si>
     <t>off</t>
   </si>
   <si>
-    <t>Product_Summary_Sorting_on_the_Product_Summary_[ANDROID]</t>
-  </si>
-  <si>
-    <t>C70781</t>
-  </si>
-  <si>
-    <t>Product_Summary-Edit_Product_view-edit_name_of_account-invalid_[MOB_ANDROID]</t>
-  </si>
-  <si>
-    <t>C70782</t>
-  </si>
-  <si>
     <t>Product_Summary-Edit_Product_view-edit_name_of_account-invalid_[MOB_ANDROID]_6</t>
   </si>
   <si>
@@ -1074,6 +1074,90 @@
     <t>C70950</t>
   </si>
   <si>
+    <t>Authentication_Mobile_Login_Forgot_PIN_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70951</t>
+  </si>
+  <si>
+    <t>Domestic_Payments_Budzetski_Non_Urgent_Payment_Model97_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70952</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Filter_By_Date_Date_Picker_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70953</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Filter_Filter_By_Type_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70954</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Filter_By_Amount_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70955</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Filter_By_Date_Date_Picker_Invalid_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70956</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Filter_Multiple_Filter_Invalid_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70957</t>
+  </si>
+  <si>
+    <t>Savings_Accounts_Transactions_Search_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70958</t>
+  </si>
+  <si>
+    <t>Credit_Cards_Transactions_Filter_By_Date_Predefined_Date_Range_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70959</t>
+  </si>
+  <si>
+    <t>Loan_Accounts_Header_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70960</t>
+  </si>
+  <si>
+    <t>Payments-Domestic_Payments_Input_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70961</t>
+  </si>
+  <si>
+    <t>Manage_Products_Favorite_account_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70962</t>
+  </si>
+  <si>
+    <t>Manage_Products_Favorite_account_[MOB_ANDROID]-Removal_Of_The_Favorite_Account</t>
+  </si>
+  <si>
+    <t>C70963</t>
+  </si>
+  <si>
+    <t>Credit_Cards-Transactions-Filter-Filter_By_Status_[MOB_ANDROID]</t>
+  </si>
+  <si>
+    <t>C70964</t>
+  </si>
+  <si>
     <t>Automated Test Names</t>
   </si>
   <si>
@@ -1084,9 +1168,6 @@
   </si>
   <si>
     <t>Payments_Domestic_Payments_Internal_Urgent_Payment_[MOB_ANDROID]</t>
-  </si>
-  <si>
-    <t>Domestic_Payments_Budzetski_Non_Urgent_Payment_Model97_[MOB_ANDROID]</t>
   </si>
   <si>
     <t>Manage_Products_Nickname_Product_[MOB_ANDROID]</t>
@@ -1819,7 +1900,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1846,7 +1927,11 @@
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2258,7 +2343,7 @@
         <v>12</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="1" spans="1:7">
@@ -2266,10 +2351,10 @@
         <v>7</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>10</v>
@@ -2289,22 +2374,22 @@
         <v>7</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>20</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="1" spans="1:7">
@@ -2327,7 +2412,7 @@
         <v>12</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="1" spans="1:7">
@@ -2350,7 +2435,7 @@
         <v>12</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" customFormat="1" spans="1:7">
@@ -2373,7 +2458,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="1" spans="1:7">
@@ -2396,7 +2481,7 @@
         <v>12</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" customFormat="1" spans="1:7">
@@ -2419,7 +2504,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="1" spans="1:7">
@@ -2442,7 +2527,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="1" spans="1:7">
@@ -2465,7 +2550,7 @@
         <v>12</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="1" spans="1:7">
@@ -2488,7 +2573,7 @@
         <v>12</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="1" spans="1:7">
@@ -2511,7 +2596,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="1" spans="1:7">
@@ -2534,7 +2619,7 @@
         <v>12</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" customFormat="1" spans="1:7">
@@ -2557,7 +2642,7 @@
         <v>12</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="1" spans="1:7">
@@ -2580,7 +2665,7 @@
         <v>12</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" customFormat="1" spans="1:7">
@@ -2603,7 +2688,7 @@
         <v>12</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" customFormat="1" spans="1:7">
@@ -2626,7 +2711,7 @@
         <v>12</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" customFormat="1" spans="1:7">
@@ -2649,7 +2734,7 @@
         <v>12</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" customFormat="1" spans="1:7">
@@ -2672,7 +2757,7 @@
         <v>12</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="1" spans="1:7">
@@ -2695,7 +2780,7 @@
         <v>12</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" customFormat="1" spans="1:7">
@@ -2718,7 +2803,7 @@
         <v>12</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" customFormat="1" spans="1:7">
@@ -2741,7 +2826,7 @@
         <v>12</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" customFormat="1" spans="1:7">
@@ -2764,7 +2849,7 @@
         <v>12</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" customFormat="1" spans="1:7">
@@ -2787,7 +2872,7 @@
         <v>12</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" customFormat="1" spans="1:7">
@@ -2810,7 +2895,7 @@
         <v>12</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" customFormat="1" spans="1:7">
@@ -2833,7 +2918,7 @@
         <v>12</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" customFormat="1" spans="1:7">
@@ -2856,7 +2941,7 @@
         <v>12</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" customFormat="1" spans="1:7">
@@ -2879,7 +2964,7 @@
         <v>12</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" customFormat="1" spans="1:7">
@@ -2902,7 +2987,7 @@
         <v>12</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" customFormat="1" spans="1:7">
@@ -2925,7 +3010,7 @@
         <v>12</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" customFormat="1" spans="1:7">
@@ -2971,7 +3056,7 @@
         <v>12</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35" customFormat="1" spans="1:7">
@@ -3017,7 +3102,7 @@
         <v>12</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" customFormat="1" spans="1:7">
@@ -3040,7 +3125,7 @@
         <v>12</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" customFormat="1" spans="1:7">
@@ -3086,7 +3171,7 @@
         <v>12</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" customFormat="1" spans="1:7">
@@ -3132,7 +3217,7 @@
         <v>12</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" customFormat="1" spans="1:7">
@@ -3155,7 +3240,7 @@
         <v>12</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" customFormat="1" spans="1:7">
@@ -3178,7 +3263,7 @@
         <v>12</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" customFormat="1" spans="1:7">
@@ -3201,7 +3286,7 @@
         <v>12</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" customFormat="1" spans="1:7">
@@ -3224,7 +3309,7 @@
         <v>12</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" customFormat="1" spans="1:7">
@@ -3247,7 +3332,7 @@
         <v>12</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" customFormat="1" spans="1:7">
@@ -3293,7 +3378,7 @@
         <v>12</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" customFormat="1" spans="1:7">
@@ -3316,7 +3401,7 @@
         <v>12</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" customFormat="1" spans="1:7">
@@ -3339,7 +3424,7 @@
         <v>12</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" customFormat="1" spans="1:7">
@@ -3385,7 +3470,7 @@
         <v>12</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" customFormat="1" spans="1:7">
@@ -3408,7 +3493,7 @@
         <v>12</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="54" customFormat="1" spans="1:7">
@@ -3431,7 +3516,7 @@
         <v>12</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="55" customFormat="1" spans="1:7">
@@ -3454,7 +3539,7 @@
         <v>12</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56" customFormat="1" spans="1:7">
@@ -3500,7 +3585,7 @@
         <v>12</v>
       </c>
       <c r="G57" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58" customFormat="1" spans="1:7">
@@ -3523,7 +3608,7 @@
         <v>12</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="59" customFormat="1" spans="1:7">
@@ -3546,7 +3631,7 @@
         <v>12</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="60" customFormat="1" spans="1:7">
@@ -3569,7 +3654,7 @@
         <v>12</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="61" customFormat="1" spans="1:7">
@@ -3592,7 +3677,7 @@
         <v>12</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="62" customFormat="1" spans="1:7">
@@ -3615,7 +3700,7 @@
         <v>12</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63" customFormat="1" spans="1:7">
@@ -3638,7 +3723,7 @@
         <v>12</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="64" customFormat="1" spans="1:7">
@@ -3661,7 +3746,7 @@
         <v>12</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="65" customFormat="1" spans="1:7">
@@ -3684,7 +3769,7 @@
         <v>12</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66" customFormat="1" spans="1:7">
@@ -3707,7 +3792,7 @@
         <v>12</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="67" customFormat="1" spans="1:7">
@@ -3730,7 +3815,7 @@
         <v>12</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="68" customFormat="1" spans="1:7">
@@ -3753,7 +3838,7 @@
         <v>12</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="69" customFormat="1" spans="1:7">
@@ -3776,7 +3861,7 @@
         <v>12</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="70" customFormat="1" spans="1:7">
@@ -3799,7 +3884,7 @@
         <v>12</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="71" customFormat="1" spans="1:7">
@@ -3868,7 +3953,7 @@
         <v>12</v>
       </c>
       <c r="G73" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="74" customFormat="1" spans="1:7">
@@ -3891,7 +3976,7 @@
         <v>12</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="75" customFormat="1" spans="1:7">
@@ -3914,7 +3999,7 @@
         <v>12</v>
       </c>
       <c r="G75" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76" customFormat="1" spans="1:7">
@@ -3937,7 +4022,7 @@
         <v>12</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="77" customFormat="1" spans="1:7">
@@ -3960,7 +4045,7 @@
         <v>12</v>
       </c>
       <c r="G77" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78" customFormat="1" spans="1:7">
@@ -4006,7 +4091,7 @@
         <v>12</v>
       </c>
       <c r="G79" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="80" customFormat="1" spans="1:7">
@@ -4052,7 +4137,7 @@
         <v>12</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="82" customFormat="1" spans="1:7">
@@ -4075,7 +4160,7 @@
         <v>12</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="83" customFormat="1" spans="1:7">
@@ -4098,7 +4183,7 @@
         <v>12</v>
       </c>
       <c r="G83" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="84" customFormat="1" spans="1:7">
@@ -4121,7 +4206,7 @@
         <v>12</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="85" customFormat="1" spans="1:7">
@@ -4236,7 +4321,7 @@
         <v>12</v>
       </c>
       <c r="G89" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="90" customFormat="1" spans="1:7">
@@ -4259,7 +4344,7 @@
         <v>12</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="91" customFormat="1" spans="1:7">
@@ -4328,7 +4413,7 @@
         <v>12</v>
       </c>
       <c r="G93" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="94" customFormat="1" spans="1:7">
@@ -4351,7 +4436,7 @@
         <v>12</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="95" customFormat="1" spans="1:7">
@@ -4374,7 +4459,7 @@
         <v>12</v>
       </c>
       <c r="G95" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="96" customFormat="1" spans="1:7">
@@ -4397,7 +4482,7 @@
         <v>12</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97" customFormat="1" spans="1:7">
@@ -4420,7 +4505,7 @@
         <v>12</v>
       </c>
       <c r="G97" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98" customFormat="1" spans="1:7">
@@ -4466,7 +4551,7 @@
         <v>12</v>
       </c>
       <c r="G99" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="100" customFormat="1" spans="1:7">
@@ -4512,7 +4597,7 @@
         <v>12</v>
       </c>
       <c r="G101" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="102" customFormat="1" spans="1:7">
@@ -4535,7 +4620,7 @@
         <v>12</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="103" customFormat="1" spans="1:7">
@@ -4558,7 +4643,7 @@
         <v>12</v>
       </c>
       <c r="G103" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="104" customFormat="1" spans="1:7">
@@ -4581,7 +4666,7 @@
         <v>12</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="105" customFormat="1" spans="1:7">
@@ -4604,7 +4689,7 @@
         <v>12</v>
       </c>
       <c r="G105" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="106" customFormat="1" spans="1:7">
@@ -4627,7 +4712,7 @@
         <v>12</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="107" customFormat="1" spans="1:7">
@@ -4650,7 +4735,7 @@
         <v>12</v>
       </c>
       <c r="G107" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="108" customFormat="1" spans="1:7">
@@ -4673,7 +4758,7 @@
         <v>12</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="109" customFormat="1" spans="1:7">
@@ -4949,7 +5034,7 @@
         <v>12</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="121" customFormat="1" spans="1:7">
@@ -4972,7 +5057,7 @@
         <v>12</v>
       </c>
       <c r="G121" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="122" customFormat="1" spans="1:7">
@@ -6000,7 +6085,7 @@
       <c r="D166" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E166" s="7" t="s">
+      <c r="E166" s="14" t="s">
         <v>11</v>
       </c>
       <c r="F166" s="6" t="s">
@@ -6029,7 +6114,7 @@
       <c r="F167" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G167" s="14" t="s">
+      <c r="G167" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -6052,7 +6137,7 @@
       <c r="F168" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G168" s="14" t="s">
+      <c r="G168" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -6075,7 +6160,7 @@
       <c r="F169" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G169" s="14" t="s">
+      <c r="G169" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -6098,7 +6183,7 @@
       <c r="F170" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G170" s="14" t="s">
+      <c r="G170" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -6121,7 +6206,7 @@
       <c r="F171" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G171" s="14" t="s">
+      <c r="G171" s="15" t="s">
         <v>13</v>
       </c>
     </row>
@@ -6144,135 +6229,331 @@
       <c r="F172" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G172" s="14" t="s">
+      <c r="G172" s="15" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="173" customFormat="1" spans="1:7">
-      <c r="A173" s="6"/>
-      <c r="B173" s="6"/>
-      <c r="C173" s="6"/>
-      <c r="D173" s="6"/>
-      <c r="E173" s="6"/>
-      <c r="F173" s="8"/>
-      <c r="G173" s="6"/>
+      <c r="A173" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B173" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="C173" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="D173" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E173" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F173" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G173" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="174" customFormat="1" spans="1:7">
-      <c r="A174" s="6"/>
-      <c r="B174" s="6"/>
-      <c r="C174" s="6"/>
-      <c r="D174" s="6"/>
-      <c r="E174" s="6"/>
-      <c r="F174" s="8"/>
-      <c r="G174" s="6"/>
+      <c r="A174" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B174" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="C174" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="D174" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E174" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F174" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G174" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="175" customFormat="1" spans="1:7">
-      <c r="A175" s="6"/>
-      <c r="B175" s="6"/>
-      <c r="C175" s="6"/>
-      <c r="D175" s="6"/>
-      <c r="E175" s="6"/>
-      <c r="F175" s="8"/>
-      <c r="G175" s="6"/>
+      <c r="A175" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B175" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C175" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="D175" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E175" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F175" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G175" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="176" customFormat="1" spans="1:7">
-      <c r="A176" s="6"/>
-      <c r="B176" s="6"/>
-      <c r="C176" s="6"/>
-      <c r="D176" s="6"/>
-      <c r="E176" s="6"/>
-      <c r="F176" s="8"/>
-      <c r="G176" s="6"/>
+      <c r="A176" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B176" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="C176" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="D176" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E176" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F176" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G176" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="177" customFormat="1" spans="1:7">
-      <c r="A177" s="6"/>
-      <c r="B177" s="6"/>
-      <c r="C177" s="6"/>
-      <c r="D177" s="6"/>
-      <c r="E177" s="6"/>
-      <c r="F177" s="8"/>
-      <c r="G177" s="6"/>
+      <c r="A177" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B177" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="C177" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="D177" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E177" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F177" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G177" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="178" customFormat="1" spans="1:7">
-      <c r="A178" s="6"/>
-      <c r="B178" s="6"/>
-      <c r="C178" s="6"/>
-      <c r="D178" s="6"/>
-      <c r="E178" s="6"/>
-      <c r="F178" s="8"/>
-      <c r="G178" s="6"/>
+      <c r="A178" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B178" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="C178" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="D178" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E178" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F178" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G178" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="179" customFormat="1" spans="1:7">
-      <c r="A179" s="6"/>
-      <c r="B179" s="6"/>
-      <c r="C179" s="6"/>
-      <c r="D179" s="6"/>
-      <c r="E179" s="6"/>
-      <c r="F179" s="8"/>
-      <c r="G179" s="6"/>
+      <c r="A179" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B179" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="C179" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="D179" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E179" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F179" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G179" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="180" customFormat="1" spans="1:7">
-      <c r="A180" s="6"/>
-      <c r="B180" s="6"/>
-      <c r="C180" s="6"/>
-      <c r="D180" s="6"/>
-      <c r="E180" s="6"/>
-      <c r="F180" s="8"/>
-      <c r="G180" s="6"/>
+      <c r="A180" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B180" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="C180" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="D180" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E180" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F180" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G180" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="181" customFormat="1" spans="1:7">
-      <c r="A181" s="6"/>
-      <c r="B181" s="6"/>
-      <c r="C181" s="6"/>
-      <c r="D181" s="6"/>
-      <c r="E181" s="6"/>
-      <c r="F181" s="8"/>
-      <c r="G181" s="6"/>
+      <c r="A181" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B181" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C181" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="D181" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E181" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F181" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G181" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="182" customFormat="1" spans="1:7">
-      <c r="A182" s="6"/>
-      <c r="B182" s="6"/>
-      <c r="C182" s="6"/>
-      <c r="D182" s="6"/>
-      <c r="E182" s="6"/>
-      <c r="F182" s="8"/>
-      <c r="G182" s="6"/>
+      <c r="A182" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B182" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C182" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="D182" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E182" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F182" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G182" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="183" customFormat="1" spans="1:7">
-      <c r="A183" s="6"/>
-      <c r="B183" s="6"/>
-      <c r="C183" s="6"/>
-      <c r="D183" s="6"/>
-      <c r="E183" s="6"/>
-      <c r="F183" s="8"/>
-      <c r="G183" s="6"/>
+      <c r="A183" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B183" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C183" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="D183" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E183" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F183" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G183" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="184" customFormat="1" spans="1:7">
-      <c r="A184" s="6"/>
-      <c r="B184" s="6"/>
-      <c r="C184" s="6"/>
-      <c r="D184" s="6"/>
-      <c r="E184" s="6"/>
-      <c r="F184" s="8"/>
-      <c r="G184" s="6"/>
+      <c r="A184" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B184" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C184" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="D184" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E184" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F184" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G184" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="185" customFormat="1" spans="1:7">
-      <c r="A185" s="6"/>
-      <c r="B185" s="6"/>
-      <c r="C185" s="6"/>
-      <c r="D185" s="6"/>
-      <c r="E185" s="6"/>
-      <c r="F185" s="8"/>
-      <c r="G185" s="6"/>
+      <c r="A185" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B185" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="C185" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="D185" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E185" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F185" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G185" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="186" customFormat="1" spans="1:7">
-      <c r="A186" s="6"/>
-      <c r="B186" s="6"/>
-      <c r="C186" s="6"/>
-      <c r="D186" s="6"/>
-      <c r="E186" s="6"/>
-      <c r="F186" s="8"/>
-      <c r="G186" s="6"/>
+      <c r="A186" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B186" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="C186" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="D186" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E186" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F186" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G186" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="187" customFormat="1" spans="1:7">
       <c r="A187" s="6"/>
@@ -6608,7 +6889,7 @@
       <c r="G223" s="6"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G171" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G186" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="C$1:C$1048576">
@@ -6636,7 +6917,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="15.15" spans="1:4">
       <c r="A1" s="2" t="s">
-        <v>347</v>
+        <v>375</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -6644,7 +6925,7 @@
     </row>
     <row r="2" s="1" customFormat="1" ht="15.15" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -6772,7 +7053,7 @@
     </row>
     <row r="18" s="1" customFormat="1" ht="15.15" spans="1:4">
       <c r="A18" s="3" t="s">
-        <v>348</v>
+        <v>376</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -6788,7 +7069,7 @@
     </row>
     <row r="20" s="1" customFormat="1" ht="15.15" spans="1:4">
       <c r="A20" s="3" t="s">
-        <v>349</v>
+        <v>377</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -6900,7 +7181,7 @@
     </row>
     <row r="34" s="1" customFormat="1" ht="15.15" spans="1:4">
       <c r="A34" s="3" t="s">
-        <v>350</v>
+        <v>378</v>
       </c>
       <c r="B34"/>
       <c r="C34"/>
@@ -6983,7 +7264,7 @@
     </row>
     <row r="47" ht="15.15" spans="1:4">
       <c r="A47" s="3" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="48" ht="15.15" spans="1:4">
@@ -7023,7 +7304,7 @@
     </row>
     <row r="55" ht="15.15" spans="1:1">
       <c r="A55" s="3" t="s">
-        <v>352</v>
+        <v>379</v>
       </c>
     </row>
     <row r="56" ht="15.15" spans="1:1">

</xml_diff>